<commit_message>
initial for dq 1-5
</commit_message>
<xml_diff>
--- a/gu_in/Quest.edf/QuestDesc.xlsx
+++ b/gu_in/Quest.edf/QuestDesc.xlsx
@@ -3,14 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286CD662-02AD-4F19-BD22-AB1204EA1252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0899A213-4319-4C8E-BDBB-5F1BC69A7729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QDescCli" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>